<commit_message>
update one8 discount rules
</commit_message>
<xml_diff>
--- a/one8_discount_rules.xlsx
+++ b/one8_discount_rules.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="30">
   <si>
     <t>category</t>
   </si>
@@ -63,6 +63,48 @@
   </si>
   <si>
     <t xml:space="preserve">2526 BURTON [AK] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2425 DIMITO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2526 DIMITO </t>
+  </si>
+  <si>
+    <t>滑雪板</t>
+  </si>
+  <si>
+    <t>2526 BURTON</t>
+  </si>
+  <si>
+    <t>2425 BURTON</t>
+  </si>
+  <si>
+    <t>滑雪鞋</t>
+  </si>
+  <si>
+    <t>2526 BURTON STEP ON</t>
+  </si>
+  <si>
+    <t>2526 BURTON KIDS STEP ON</t>
+  </si>
+  <si>
+    <t>2526 BURTON KIDS</t>
+  </si>
+  <si>
+    <t>2425 BURTON KIDS STEP ON</t>
+  </si>
+  <si>
+    <t>2425 BURTON KIDS</t>
+  </si>
+  <si>
+    <t>2425 FLUX</t>
+  </si>
+  <si>
+    <t>2526 FLUX</t>
+  </si>
+  <si>
+    <t>2526 FLUX STEP ON</t>
   </si>
 </sst>
 </file>
@@ -75,13 +117,25 @@
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFA0A0A0"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF757575"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="8.25"/>
@@ -544,154 +598,156 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1038,8 +1094,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="6"/>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
     <col min="2" max="2" width="27.6153846153846" customWidth="1"/>
     <col min="3" max="3" width="14.3846153846154" customWidth="1"/>
@@ -1111,7 +1167,7 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="3">
         <v>200</v>
       </c>
     </row>
@@ -1183,6 +1239,380 @@
         <v>1</v>
       </c>
       <c r="F7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6">
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>0.5</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6">
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9">
+        <v>0.6</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>0.6</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>0.5</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12">
+        <v>0.6</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13">
+        <v>0.6</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14">
+        <v>0.65</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15">
+        <v>0.65</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16">
+        <v>0.6</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17">
+        <v>0.6</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>0.7</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19">
+        <v>0.7</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>7</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21">
+        <v>0.65</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22">
+        <v>0.65</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23">
+        <v>0.65</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24">
+        <v>0.55</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25">
+        <v>0.6</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26">
+        <v>0.65</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update one8 discount matching rules
</commit_message>
<xml_diff>
--- a/one8_discount_rules.xlsx
+++ b/one8_discount_rules.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="34">
   <si>
     <t>category</t>
   </si>
@@ -65,6 +65,9 @@
     <t>2526 NITRO</t>
   </si>
   <si>
+    <t>滑雪服</t>
+  </si>
+  <si>
     <t xml:space="preserve">2526 BURTON [AK] </t>
   </si>
   <si>
@@ -111,6 +114,12 @@
   </si>
   <si>
     <t>2526 FLUX STEP ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2425 BURTON [AK] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2526 BURTON KIDS </t>
   </si>
 </sst>
 </file>
@@ -1099,8 +1108,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:G26"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
     <col min="2" max="2" width="27.6153846153846" customWidth="1"/>
@@ -1134,7 +1143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" hidden="1" spans="1:7">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1157,7 +1166,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" hidden="1" spans="1:6">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1177,7 +1186,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" hidden="1" spans="1:6">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1197,7 +1206,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="2:6">
+    <row r="5" hidden="1" spans="2:6">
       <c r="B5" t="s">
         <v>13</v>
       </c>
@@ -1214,7 +1223,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
+    <row r="6" hidden="1" spans="2:6">
       <c r="B6" t="s">
         <v>14</v>
       </c>
@@ -1231,9 +1240,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -1248,9 +1260,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="2:6">
+    <row r="8" hidden="1" spans="2:6">
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
         <v>9</v>
@@ -1265,9 +1277,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="2:6">
+    <row r="9" hidden="1" spans="2:6">
       <c r="B9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
         <v>9</v>
@@ -1284,10 +1296,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
@@ -1304,10 +1316,10 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -1327,7 +1339,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
@@ -1344,10 +1356,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
@@ -1367,7 +1379,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
         <v>9</v>
@@ -1384,10 +1396,10 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
@@ -1407,7 +1419,7 @@
         <v>7</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
         <v>9</v>
@@ -1424,10 +1436,10 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
         <v>9</v>
@@ -1447,7 +1459,7 @@
         <v>7</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" t="s">
         <v>9</v>
@@ -1464,10 +1476,10 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
@@ -1484,10 +1496,10 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
         <v>9</v>
@@ -1507,7 +1519,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
         <v>9</v>
@@ -1524,10 +1536,10 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
@@ -1544,10 +1556,10 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
@@ -1562,12 +1574,12 @@
         <v>250</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" hidden="1" spans="1:6">
       <c r="A24" t="s">
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C24" t="s">
         <v>9</v>
@@ -1582,12 +1594,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" hidden="1" spans="1:6">
       <c r="A25" t="s">
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
         <v>9</v>
@@ -1602,12 +1614,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" hidden="1" spans="1:6">
       <c r="A26" t="s">
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
         <v>9</v>
@@ -1619,11 +1631,84 @@
         <v>1</v>
       </c>
       <c r="F26">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27">
+        <v>0.55</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
         <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28">
+        <v>0.6</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29">
+        <v>0.65</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G26">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="2425 BURTON KIDS"/>
+        <filter val="2526 BURTON KIDS"/>
+        <filter val="2526 BURTON [AK]"/>
+        <filter val="2425 BURTON"/>
+        <filter val="2526 BURTON"/>
+        <filter val="2526 BURTON STEP ON"/>
+        <filter val="2425 BURTON STEP ON"/>
+        <filter val="2425 BURTON KIDS STEP ON"/>
+        <filter val="2526 BURTON KIDS STEP ON"/>
+      </filters>
+    </filterColumn>
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>